<commit_message>
Update NY gaming data - Thu Sep 17 17:00:46 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -52,12 +52,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -201,12 +201,24 @@
     <xf numFmtId="3" fontId="3" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -219,12 +231,6 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -240,18 +246,18 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -261,19 +267,16 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -780,670 +783,634 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>9/6/2026</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="n">
-        <v>171492780</v>
-      </c>
-      <c r="C3" s="10" t="n">
-        <v>16692306</v>
-      </c>
-      <c r="D3" s="11" t="n">
-        <v>0.0973353280528778</v>
-      </c>
+          <t>9/13/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n"/>
+      <c r="C3" s="10" t="n"/>
+      <c r="D3" s="11" t="n"/>
       <c r="E3" s="9" t="n">
-        <v>167953524</v>
+        <v>224469222</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>16892923</v>
-      </c>
-      <c r="G3" s="11" t="n">
-        <v>0.1005809380933263</v>
+        <v>8347252</v>
+      </c>
+      <c r="G3" s="12" t="n">
+        <v>0.03718662191469609</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>34668902</v>
+        <v>35436082</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>3546293</v>
-      </c>
-      <c r="J3" s="11" t="n">
-        <v>0.1022903177031681</v>
-      </c>
-      <c r="K3" s="9" t="n">
-        <v>56782523</v>
-      </c>
-      <c r="L3" s="10" t="n">
-        <v>3258000</v>
-      </c>
-      <c r="M3" s="11" t="n">
-        <v>0.05737680941017714</v>
-      </c>
+        <v>966974</v>
+      </c>
+      <c r="J3" s="12" t="n">
+        <v>0.02728783616653782</v>
+      </c>
+      <c r="K3" s="9" t="n"/>
+      <c r="L3" s="10" t="n"/>
+      <c r="M3" s="11" t="n"/>
       <c r="N3" s="9" t="n">
-        <v>483313174</v>
+        <v>263117002</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>44849147</v>
-      </c>
-      <c r="P3" s="11" t="n">
-        <v>0.09279520901286253</v>
+        <v>9418255</v>
+      </c>
+      <c r="P3" s="12" t="n">
+        <v>0.03579493160232945</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>-16%</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>+273%</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>+756bps</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>-3%</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>+16%</t>
-        </is>
-      </c>
-      <c r="G4" s="15" t="inlineStr">
-        <is>
-          <t>+168bps</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>-6%</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>+87%</t>
-        </is>
-      </c>
-      <c r="J4" s="15" t="inlineStr">
-        <is>
-          <t>+509bps</t>
-        </is>
-      </c>
-      <c r="K4" s="16" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="L4" s="17" t="inlineStr">
-        <is>
-          <t>-45%</t>
-        </is>
-      </c>
-      <c r="M4" s="18" t="inlineStr">
-        <is>
-          <t>-567bps</t>
-        </is>
-      </c>
-      <c r="N4" s="13" t="inlineStr">
-        <is>
-          <t>-8%</t>
-        </is>
-      </c>
-      <c r="O4" s="14" t="inlineStr">
-        <is>
-          <t>+47%</t>
-        </is>
-      </c>
-      <c r="P4" s="15" t="inlineStr">
-        <is>
-          <t>+349bps</t>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>+28%</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>-65%</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>-1005bps</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="inlineStr">
+        <is>
+          <t>+11%</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>-61%</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>-508bps</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="n"/>
+      <c r="L4" s="15" t="n"/>
+      <c r="M4" s="16" t="n"/>
+      <c r="N4" s="20" t="inlineStr">
+        <is>
+          <t>-51%</t>
+        </is>
+      </c>
+      <c r="O4" s="18" t="inlineStr">
+        <is>
+          <t>-83%</t>
+        </is>
+      </c>
+      <c r="P4" s="19" t="inlineStr">
+        <is>
+          <t>-707bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>8/30/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>149527600</v>
-      </c>
-      <c r="C5" s="21" t="n">
-        <v>12079306</v>
-      </c>
-      <c r="D5" s="22" t="n">
-        <v>0.08078311963811363</v>
-      </c>
-      <c r="E5" s="20" t="n">
-        <v>146777769</v>
-      </c>
-      <c r="F5" s="21" t="n">
-        <v>15874317</v>
-      </c>
-      <c r="G5" s="22" t="n">
-        <v>0.1081520526449751</v>
-      </c>
-      <c r="H5" s="20" t="n">
-        <v>29155390</v>
-      </c>
-      <c r="I5" s="21" t="n">
-        <v>2727869</v>
-      </c>
-      <c r="J5" s="22" t="n">
-        <v>0.09356311131492324</v>
-      </c>
-      <c r="K5" s="20" t="n">
-        <v>52848942</v>
-      </c>
-      <c r="L5" s="21" t="n">
-        <v>5061346</v>
-      </c>
-      <c r="M5" s="22" t="n">
-        <v>0.09577005344780601</v>
-      </c>
-      <c r="N5" s="20" t="n">
-        <v>420285714</v>
-      </c>
-      <c r="O5" s="21" t="n">
-        <v>39300665</v>
-      </c>
-      <c r="P5" s="22" t="n">
-        <v>0.09350940013154956</v>
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>9/6/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="n">
+        <v>171492780</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>16692306</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>0.0973353280528778</v>
+      </c>
+      <c r="E5" s="22" t="n">
+        <v>167953524</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <v>16892923</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <v>0.1005809380933263</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>34668902</v>
+      </c>
+      <c r="I5" s="23" t="n">
+        <v>3546293</v>
+      </c>
+      <c r="J5" s="24" t="n">
+        <v>0.1022903177031681</v>
+      </c>
+      <c r="K5" s="22" t="n">
+        <v>56782523</v>
+      </c>
+      <c r="L5" s="23" t="n">
+        <v>3258000</v>
+      </c>
+      <c r="M5" s="24" t="n">
+        <v>0.05737680941017714</v>
+      </c>
+      <c r="N5" s="22" t="n">
+        <v>483313174</v>
+      </c>
+      <c r="O5" s="23" t="n">
+        <v>44849147</v>
+      </c>
+      <c r="P5" s="24" t="n">
+        <v>0.09279520901286253</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>-10%</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="inlineStr">
-        <is>
-          <t>-39%</t>
-        </is>
-      </c>
-      <c r="D6" s="26" t="inlineStr">
-        <is>
-          <t>-392bps</t>
-        </is>
-      </c>
-      <c r="E6" s="24" t="inlineStr">
-        <is>
-          <t>-4%</t>
-        </is>
-      </c>
-      <c r="F6" s="25" t="inlineStr">
-        <is>
-          <t>-27%</t>
-        </is>
-      </c>
-      <c r="G6" s="26" t="inlineStr">
-        <is>
-          <t>-338bps</t>
-        </is>
-      </c>
-      <c r="H6" s="24" t="inlineStr">
-        <is>
-          <t>-25%</t>
-        </is>
-      </c>
-      <c r="I6" s="25" t="inlineStr">
-        <is>
-          <t>-37%</t>
-        </is>
-      </c>
-      <c r="J6" s="26" t="inlineStr">
-        <is>
-          <t>-186bps</t>
-        </is>
-      </c>
-      <c r="K6" s="24" t="inlineStr">
-        <is>
-          <t>-64%</t>
-        </is>
-      </c>
-      <c r="L6" s="25" t="inlineStr">
-        <is>
-          <t>-66%</t>
-        </is>
-      </c>
-      <c r="M6" s="26" t="inlineStr">
-        <is>
-          <t>-57bps</t>
-        </is>
-      </c>
-      <c r="N6" s="24" t="inlineStr">
-        <is>
-          <t>-25%</t>
-        </is>
-      </c>
-      <c r="O6" s="25" t="inlineStr">
-        <is>
-          <t>-41%</t>
-        </is>
-      </c>
-      <c r="P6" s="26" t="inlineStr">
-        <is>
-          <t>-259bps</t>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>-16%</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>+273%</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>+756bps</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>-3%</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>+16%</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>+168bps</t>
+        </is>
+      </c>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>-6%</t>
+        </is>
+      </c>
+      <c r="I6" s="27" t="inlineStr">
+        <is>
+          <t>+87%</t>
+        </is>
+      </c>
+      <c r="J6" s="28" t="inlineStr">
+        <is>
+          <t>+509bps</t>
+        </is>
+      </c>
+      <c r="K6" s="29" t="inlineStr">
+        <is>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="L6" s="30" t="inlineStr">
+        <is>
+          <t>-45%</t>
+        </is>
+      </c>
+      <c r="M6" s="31" t="inlineStr">
+        <is>
+          <t>-567bps</t>
+        </is>
+      </c>
+      <c r="N6" s="26" t="inlineStr">
+        <is>
+          <t>-8%</t>
+        </is>
+      </c>
+      <c r="O6" s="27" t="inlineStr">
+        <is>
+          <t>+47%</t>
+        </is>
+      </c>
+      <c r="P6" s="28" t="inlineStr">
+        <is>
+          <t>+349bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>8/23/2026</t>
+          <t>8/30/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>137507207</v>
+        <v>149527600</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>10643451</v>
-      </c>
-      <c r="D7" s="11" t="n">
-        <v>0.07740285932794781</v>
+        <v>12079306</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>0.08078311963811363</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>132060011</v>
+        <v>146777769</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>10710519</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>0.08110342350342527</v>
+        <v>15874317</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>0.1081520526449751</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>24881322</v>
+        <v>29155390</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>1911178</v>
-      </c>
-      <c r="J7" s="11" t="n">
-        <v>0.07681175461657544</v>
+        <v>2727869</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>0.09356311131492324</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>47701558</v>
+        <v>52848942</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>3476356</v>
-      </c>
-      <c r="M7" s="11" t="n">
-        <v>0.07287720036314117</v>
+        <v>5061346</v>
+      </c>
+      <c r="M7" s="12" t="n">
+        <v>0.09577005344780601</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>381646903</v>
+        <v>420285714</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>30506351</v>
-      </c>
-      <c r="P7" s="11" t="n">
-        <v>0.07993344308626553</v>
+        <v>39300665</v>
+      </c>
+      <c r="P7" s="12" t="n">
+        <v>0.09350940013154956</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>+4%</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>-31%</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>-395bps</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>+5%</t>
-        </is>
-      </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>-10%</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>-39%</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>-392bps</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>-4%</t>
         </is>
       </c>
-      <c r="G8" s="18" t="inlineStr">
-        <is>
-          <t>-78bps</t>
-        </is>
-      </c>
-      <c r="H8" s="13" t="inlineStr">
-        <is>
-          <t>-11%</t>
-        </is>
-      </c>
-      <c r="I8" s="17" t="inlineStr">
-        <is>
-          <t>-36%</t>
-        </is>
-      </c>
-      <c r="J8" s="18" t="inlineStr">
-        <is>
-          <t>-301bps</t>
-        </is>
-      </c>
-      <c r="K8" s="13" t="inlineStr">
-        <is>
-          <t>-78%</t>
-        </is>
-      </c>
-      <c r="L8" s="14" t="inlineStr">
-        <is>
-          <t>+688%</t>
-        </is>
-      </c>
-      <c r="M8" s="15" t="inlineStr">
-        <is>
-          <t>+708bps</t>
-        </is>
-      </c>
-      <c r="N8" s="13" t="inlineStr">
-        <is>
-          <t>-30%</t>
-        </is>
-      </c>
-      <c r="O8" s="17" t="inlineStr">
-        <is>
-          <t>-11%</t>
-        </is>
-      </c>
-      <c r="P8" s="15" t="inlineStr">
-        <is>
-          <t>+170bps</t>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>-27%</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>-338bps</t>
+        </is>
+      </c>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>-37%</t>
+        </is>
+      </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>-186bps</t>
+        </is>
+      </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>-64%</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>-66%</t>
+        </is>
+      </c>
+      <c r="M8" s="19" t="inlineStr">
+        <is>
+          <t>-57bps</t>
+        </is>
+      </c>
+      <c r="N8" s="20" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="O8" s="18" t="inlineStr">
+        <is>
+          <t>-41%</t>
+        </is>
+      </c>
+      <c r="P8" s="19" t="inlineStr">
+        <is>
+          <t>-259bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>8/16/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n">
-        <v>139804782</v>
-      </c>
-      <c r="C9" s="21" t="n">
-        <v>14936414</v>
-      </c>
-      <c r="D9" s="22" t="n">
-        <v>0.1068376473703167</v>
-      </c>
-      <c r="E9" s="20" t="n">
-        <v>128334482</v>
-      </c>
-      <c r="F9" s="21" t="n">
-        <v>16567440</v>
-      </c>
-      <c r="G9" s="22" t="n">
-        <v>0.1290957795738794</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <v>26211607</v>
-      </c>
-      <c r="I9" s="21" t="n">
-        <v>3989974</v>
-      </c>
-      <c r="J9" s="22" t="n">
-        <v>0.1522216474556482</v>
-      </c>
-      <c r="K9" s="20" t="n">
-        <v>43618315</v>
-      </c>
-      <c r="L9" s="21" t="n">
-        <v>4332991</v>
-      </c>
-      <c r="M9" s="22" t="n">
-        <v>0.09933879839237256</v>
-      </c>
-      <c r="N9" s="20" t="n">
-        <v>380789208</v>
-      </c>
-      <c r="O9" s="21" t="n">
-        <v>44525193</v>
-      </c>
-      <c r="P9" s="22" t="n">
-        <v>0.1169287155848177</v>
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>8/23/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="n">
+        <v>137507207</v>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>10643451</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>0.07740285932794781</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>132060011</v>
+      </c>
+      <c r="F9" s="23" t="n">
+        <v>10710519</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>0.08110342350342527</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <v>24881322</v>
+      </c>
+      <c r="I9" s="23" t="n">
+        <v>1911178</v>
+      </c>
+      <c r="J9" s="24" t="n">
+        <v>0.07681175461657544</v>
+      </c>
+      <c r="K9" s="22" t="n">
+        <v>47701558</v>
+      </c>
+      <c r="L9" s="23" t="n">
+        <v>3476356</v>
+      </c>
+      <c r="M9" s="24" t="n">
+        <v>0.07287720036314117</v>
+      </c>
+      <c r="N9" s="22" t="n">
+        <v>381646903</v>
+      </c>
+      <c r="O9" s="23" t="n">
+        <v>30506351</v>
+      </c>
+      <c r="P9" s="24" t="n">
+        <v>0.07993344308626553</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="27" t="inlineStr">
-        <is>
-          <t>+14%</t>
-        </is>
-      </c>
-      <c r="C10" s="28" t="inlineStr">
-        <is>
-          <t>+38%</t>
-        </is>
-      </c>
-      <c r="D10" s="29" t="inlineStr">
-        <is>
-          <t>+182bps</t>
-        </is>
-      </c>
-      <c r="E10" s="27" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="F10" s="28" t="inlineStr">
-        <is>
-          <t>+17%</t>
-        </is>
-      </c>
-      <c r="G10" s="29" t="inlineStr">
-        <is>
-          <t>+80bps</t>
-        </is>
-      </c>
-      <c r="H10" s="24" t="inlineStr">
-        <is>
-          <t>-1%</t>
-        </is>
-      </c>
-      <c r="I10" s="28" t="inlineStr">
-        <is>
-          <t>+61%</t>
-        </is>
-      </c>
-      <c r="J10" s="29" t="inlineStr">
-        <is>
-          <t>+590bps</t>
-        </is>
-      </c>
-      <c r="K10" s="24" t="inlineStr">
-        <is>
-          <t>-70%</t>
-        </is>
-      </c>
-      <c r="L10" s="28" t="inlineStr">
-        <is>
-          <t>+61%</t>
-        </is>
-      </c>
-      <c r="M10" s="29" t="inlineStr">
-        <is>
-          <t>+811bps</t>
-        </is>
-      </c>
-      <c r="N10" s="24" t="inlineStr">
-        <is>
-          <t>-17%</t>
-        </is>
-      </c>
-      <c r="O10" s="28" t="inlineStr">
-        <is>
-          <t>+34%</t>
-        </is>
-      </c>
-      <c r="P10" s="29" t="inlineStr">
-        <is>
-          <t>+441bps</t>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>+4%</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>-31%</t>
+        </is>
+      </c>
+      <c r="D10" s="31" t="inlineStr">
+        <is>
+          <t>-395bps</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>-4%</t>
+        </is>
+      </c>
+      <c r="G10" s="31" t="inlineStr">
+        <is>
+          <t>-78bps</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="I10" s="30" t="inlineStr">
+        <is>
+          <t>-36%</t>
+        </is>
+      </c>
+      <c r="J10" s="31" t="inlineStr">
+        <is>
+          <t>-301bps</t>
+        </is>
+      </c>
+      <c r="K10" s="26" t="inlineStr">
+        <is>
+          <t>-78%</t>
+        </is>
+      </c>
+      <c r="L10" s="27" t="inlineStr">
+        <is>
+          <t>+688%</t>
+        </is>
+      </c>
+      <c r="M10" s="28" t="inlineStr">
+        <is>
+          <t>+708bps</t>
+        </is>
+      </c>
+      <c r="N10" s="26" t="inlineStr">
+        <is>
+          <t>-30%</t>
+        </is>
+      </c>
+      <c r="O10" s="30" t="inlineStr">
+        <is>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="P10" s="28" t="inlineStr">
+        <is>
+          <t>+170bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>8/9/2026</t>
+          <t>8/16/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>125731438</v>
+        <v>139804782</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>11195807</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>0.08904540644798797</v>
+        <v>14936414</v>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>0.1068376473703167</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>131288243</v>
+        <v>128334482</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>14045656</v>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>0.1069833496057983</v>
+        <v>16567440</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>0.1290957795738794</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>25099261</v>
+        <v>26211607</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>3458247</v>
-      </c>
-      <c r="J11" s="11" t="n">
-        <v>0.1377828215739101</v>
+        <v>3989974</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>0.1522216474556482</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>48494523</v>
+        <v>43618315</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>4176190</v>
-      </c>
-      <c r="M11" s="11" t="n">
-        <v>0.08611673528575588</v>
+        <v>4332991</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>0.09933879839237256</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>372916925</v>
+        <v>380789208</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>36677501</v>
-      </c>
-      <c r="P11" s="11" t="n">
-        <v>0.09835300717445312</v>
+        <v>44525193</v>
+      </c>
+      <c r="P11" s="12" t="n">
+        <v>0.1169287155848177</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B12" s="31" t="inlineStr">
-        <is>
-          <t>+19%</t>
-        </is>
-      </c>
-      <c r="C12" s="32" t="inlineStr">
-        <is>
-          <t>-2%</t>
-        </is>
-      </c>
-      <c r="D12" s="33" t="inlineStr">
-        <is>
-          <t>-191bps</t>
-        </is>
-      </c>
-      <c r="E12" s="31" t="inlineStr">
-        <is>
-          <t>+16%</t>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>+14%</t>
+        </is>
+      </c>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>+38%</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>+182bps</t>
+        </is>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>+9%</t>
         </is>
       </c>
       <c r="F12" s="34" t="inlineStr">
         <is>
-          <t>+3%</t>
-        </is>
-      </c>
-      <c r="G12" s="33" t="inlineStr">
-        <is>
-          <t>-129bps</t>
-        </is>
-      </c>
-      <c r="H12" s="31" t="inlineStr">
-        <is>
-          <t>+3%</t>
+          <t>+17%</t>
+        </is>
+      </c>
+      <c r="G12" s="35" t="inlineStr">
+        <is>
+          <t>+80bps</t>
+        </is>
+      </c>
+      <c r="H12" s="36" t="inlineStr">
+        <is>
+          <t>-1%</t>
         </is>
       </c>
       <c r="I12" s="34" t="inlineStr">
         <is>
-          <t>+40%</t>
+          <t>+61%</t>
         </is>
       </c>
       <c r="J12" s="35" t="inlineStr">
         <is>
-          <t>+366bps</t>
-        </is>
-      </c>
-      <c r="K12" s="31" t="inlineStr">
-        <is>
-          <t>+48%</t>
+          <t>+590bps</t>
+        </is>
+      </c>
+      <c r="K12" s="36" t="inlineStr">
+        <is>
+          <t>-70%</t>
         </is>
       </c>
       <c r="L12" s="34" t="inlineStr">
         <is>
-          <t>+12%</t>
-        </is>
-      </c>
-      <c r="M12" s="33" t="inlineStr">
-        <is>
-          <t>-278bps</t>
-        </is>
-      </c>
-      <c r="N12" s="31" t="inlineStr">
-        <is>
-          <t>+18%</t>
+          <t>+61%</t>
+        </is>
+      </c>
+      <c r="M12" s="35" t="inlineStr">
+        <is>
+          <t>+811bps</t>
+        </is>
+      </c>
+      <c r="N12" s="36" t="inlineStr">
+        <is>
+          <t>-17%</t>
         </is>
       </c>
       <c r="O12" s="34" t="inlineStr">
         <is>
-          <t>+5%</t>
-        </is>
-      </c>
-      <c r="P12" s="33" t="inlineStr">
-        <is>
-          <t>-121bps</t>
+          <t>+34%</t>
+        </is>
+      </c>
+      <c r="P12" s="35" t="inlineStr">
+        <is>
+          <t>+441bps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NY gaming data - Thu Sep 24 20:00:55 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -52,12 +52,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -204,12 +204,57 @@
     <xf numFmtId="164" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -219,52 +264,25 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -771,670 +789,616 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>9/13/2026</t>
+          <t>9/20/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>216744126</v>
+        <v>208382110</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>4743263</v>
+        <v>14221076</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.02188415938893772</v>
-      </c>
-      <c r="E3" s="9" t="n">
-        <v>224469223</v>
-      </c>
-      <c r="F3" s="10" t="n">
-        <v>8347252</v>
-      </c>
-      <c r="G3" s="11" t="n">
-        <v>0.03718662134808566</v>
-      </c>
-      <c r="H3" s="9" t="n">
-        <v>35436082</v>
-      </c>
-      <c r="I3" s="10" t="n">
-        <v>966974</v>
-      </c>
-      <c r="J3" s="11" t="n">
-        <v>0.02728783616653782</v>
-      </c>
-      <c r="K3" s="9" t="n">
-        <v>60516979</v>
-      </c>
-      <c r="L3" s="10" t="n">
-        <v>642600</v>
-      </c>
-      <c r="M3" s="11" t="n">
-        <v>0.0106185075761961</v>
-      </c>
+        <v>0.06824518669093042</v>
+      </c>
+      <c r="E3" s="9" t="n"/>
+      <c r="F3" s="10" t="n"/>
+      <c r="G3" s="12" t="n"/>
+      <c r="H3" s="9" t="n"/>
+      <c r="I3" s="10" t="n"/>
+      <c r="J3" s="12" t="n"/>
+      <c r="K3" s="9" t="n"/>
+      <c r="L3" s="10" t="n"/>
+      <c r="M3" s="12" t="n"/>
       <c r="N3" s="9" t="n">
-        <v>594594255</v>
+        <v>219373600</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>16963048</v>
+        <v>14936716</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.02852877883927755</v>
+        <v>0.06808802882388765</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>+7%</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>-76%</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>-777bps</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>+28%</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>-65%</t>
-        </is>
-      </c>
-      <c r="G4" s="15" t="inlineStr">
-        <is>
-          <t>-1005bps</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>+11%</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>-5%</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>-37%</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>-339bps</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="18" t="n"/>
+      <c r="G4" s="19" t="n"/>
+      <c r="H4" s="17" t="n"/>
+      <c r="I4" s="18" t="n"/>
+      <c r="J4" s="19" t="n"/>
+      <c r="K4" s="17" t="n"/>
+      <c r="L4" s="18" t="n"/>
+      <c r="M4" s="19" t="n"/>
+      <c r="N4" s="14" t="inlineStr">
         <is>
           <t>-61%</t>
         </is>
       </c>
-      <c r="J4" s="15" t="inlineStr">
-        <is>
-          <t>-508bps</t>
-        </is>
-      </c>
-      <c r="K4" s="16" t="inlineStr">
-        <is>
-          <t>-8%</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="inlineStr">
-        <is>
-          <t>-88%</t>
-        </is>
-      </c>
-      <c r="M4" s="15" t="inlineStr">
-        <is>
-          <t>-732bps</t>
-        </is>
-      </c>
-      <c r="N4" s="13" t="inlineStr">
-        <is>
-          <t>+11%</t>
-        </is>
-      </c>
-      <c r="O4" s="14" t="inlineStr">
-        <is>
-          <t>-70%</t>
-        </is>
-      </c>
-      <c r="P4" s="15" t="inlineStr">
-        <is>
-          <t>-780bps</t>
+      <c r="O4" s="15" t="inlineStr">
+        <is>
+          <t>-74%</t>
+        </is>
+      </c>
+      <c r="P4" s="16" t="inlineStr">
+        <is>
+          <t>-343bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>9/6/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="n">
-        <v>171492780</v>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>16692306</v>
-      </c>
-      <c r="D5" s="20" t="n">
-        <v>0.0973353280528778</v>
-      </c>
-      <c r="E5" s="18" t="n">
-        <v>167953524</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>16892923</v>
-      </c>
-      <c r="G5" s="20" t="n">
-        <v>0.1005809380933263</v>
-      </c>
-      <c r="H5" s="18" t="n">
-        <v>34668902</v>
-      </c>
-      <c r="I5" s="19" t="n">
-        <v>3546293</v>
-      </c>
-      <c r="J5" s="20" t="n">
-        <v>0.1022903177031681</v>
-      </c>
-      <c r="K5" s="18" t="n">
-        <v>56782523</v>
-      </c>
-      <c r="L5" s="19" t="n">
-        <v>3258000</v>
-      </c>
-      <c r="M5" s="20" t="n">
-        <v>0.05737680941017714</v>
-      </c>
-      <c r="N5" s="18" t="n">
-        <v>483313174</v>
-      </c>
-      <c r="O5" s="19" t="n">
-        <v>44849147</v>
-      </c>
-      <c r="P5" s="20" t="n">
-        <v>0.09279520901286253</v>
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>9/13/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>216744126</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>4743263</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>0.02188415938893772</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>224469223</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>8347252</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>0.03718662134808566</v>
+      </c>
+      <c r="H5" s="21" t="n">
+        <v>35436082</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>966974</v>
+      </c>
+      <c r="J5" s="23" t="n">
+        <v>0.02728783616653782</v>
+      </c>
+      <c r="K5" s="21" t="n">
+        <v>60516979</v>
+      </c>
+      <c r="L5" s="22" t="n">
+        <v>642600</v>
+      </c>
+      <c r="M5" s="23" t="n">
+        <v>0.0106185075761961</v>
+      </c>
+      <c r="N5" s="21" t="n">
+        <v>594594255</v>
+      </c>
+      <c r="O5" s="22" t="n">
+        <v>16963048</v>
+      </c>
+      <c r="P5" s="23" t="n">
+        <v>0.02852877883927755</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
-        <is>
-          <t>-16%</t>
-        </is>
-      </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>+273%</t>
-        </is>
-      </c>
-      <c r="D6" s="24" t="inlineStr">
-        <is>
-          <t>+756bps</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>-3%</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="inlineStr">
-        <is>
-          <t>+16%</t>
-        </is>
-      </c>
-      <c r="G6" s="24" t="inlineStr">
-        <is>
-          <t>+168bps</t>
-        </is>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>-6%</t>
-        </is>
-      </c>
-      <c r="I6" s="23" t="inlineStr">
-        <is>
-          <t>+87%</t>
-        </is>
-      </c>
-      <c r="J6" s="24" t="inlineStr">
-        <is>
-          <t>+509bps</t>
-        </is>
-      </c>
-      <c r="K6" s="25" t="inlineStr">
-        <is>
-          <t>+9%</t>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>+7%</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>-76%</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>-777bps</t>
+        </is>
+      </c>
+      <c r="E6" s="25" t="inlineStr">
+        <is>
+          <t>+28%</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>-65%</t>
+        </is>
+      </c>
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>-1005bps</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>+11%</t>
+        </is>
+      </c>
+      <c r="I6" s="26" t="inlineStr">
+        <is>
+          <t>-61%</t>
+        </is>
+      </c>
+      <c r="J6" s="27" t="inlineStr">
+        <is>
+          <t>-508bps</t>
+        </is>
+      </c>
+      <c r="K6" s="28" t="inlineStr">
+        <is>
+          <t>-8%</t>
         </is>
       </c>
       <c r="L6" s="26" t="inlineStr">
         <is>
-          <t>-45%</t>
+          <t>-88%</t>
         </is>
       </c>
       <c r="M6" s="27" t="inlineStr">
         <is>
-          <t>-567bps</t>
-        </is>
-      </c>
-      <c r="N6" s="22" t="inlineStr">
-        <is>
-          <t>-8%</t>
-        </is>
-      </c>
-      <c r="O6" s="23" t="inlineStr">
-        <is>
-          <t>+47%</t>
-        </is>
-      </c>
-      <c r="P6" s="24" t="inlineStr">
-        <is>
-          <t>+349bps</t>
+          <t>-732bps</t>
+        </is>
+      </c>
+      <c r="N6" s="25" t="inlineStr">
+        <is>
+          <t>+11%</t>
+        </is>
+      </c>
+      <c r="O6" s="26" t="inlineStr">
+        <is>
+          <t>-70%</t>
+        </is>
+      </c>
+      <c r="P6" s="27" t="inlineStr">
+        <is>
+          <t>-780bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>8/30/2026</t>
+          <t>9/6/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>149527600</v>
+        <v>171492780</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>12079306</v>
+        <v>16692306</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.08078311963811363</v>
+        <v>0.0973353280528778</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>146777769</v>
+        <v>167953524</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>15874317</v>
+        <v>16892923</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.1081520526449751</v>
+        <v>0.1005809380933263</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>29155390</v>
+        <v>34668902</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>2727869</v>
+        <v>3546293</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.09356311131492324</v>
+        <v>0.1022903177031681</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>52848942</v>
+        <v>56782523</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>5061346</v>
+        <v>3258000</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.09577005344780601</v>
+        <v>0.05737680941017714</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>420285714</v>
+        <v>483313174</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>39300665</v>
+        <v>44849147</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.09350940013154956</v>
+        <v>0.09279520901286253</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>-10%</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>-39%</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>-392bps</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>-4%</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>-27%</t>
-        </is>
-      </c>
-      <c r="G8" s="15" t="inlineStr">
-        <is>
-          <t>-338bps</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="inlineStr">
-        <is>
-          <t>-25%</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>-37%</t>
-        </is>
-      </c>
-      <c r="J8" s="15" t="inlineStr">
-        <is>
-          <t>-186bps</t>
-        </is>
-      </c>
-      <c r="K8" s="16" t="inlineStr">
-        <is>
-          <t>-64%</t>
-        </is>
-      </c>
-      <c r="L8" s="14" t="inlineStr">
-        <is>
-          <t>-66%</t>
-        </is>
-      </c>
-      <c r="M8" s="15" t="inlineStr">
-        <is>
-          <t>-57bps</t>
-        </is>
-      </c>
-      <c r="N8" s="16" t="inlineStr">
-        <is>
-          <t>-25%</t>
-        </is>
-      </c>
-      <c r="O8" s="14" t="inlineStr">
-        <is>
-          <t>-41%</t>
-        </is>
-      </c>
-      <c r="P8" s="15" t="inlineStr">
-        <is>
-          <t>-259bps</t>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>-16%</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>+273%</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>+756bps</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>-3%</t>
+        </is>
+      </c>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>+16%</t>
+        </is>
+      </c>
+      <c r="G8" s="30" t="inlineStr">
+        <is>
+          <t>+168bps</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>-6%</t>
+        </is>
+      </c>
+      <c r="I8" s="29" t="inlineStr">
+        <is>
+          <t>+87%</t>
+        </is>
+      </c>
+      <c r="J8" s="30" t="inlineStr">
+        <is>
+          <t>+509bps</t>
+        </is>
+      </c>
+      <c r="K8" s="31" t="inlineStr">
+        <is>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>-45%</t>
+        </is>
+      </c>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>-567bps</t>
+        </is>
+      </c>
+      <c r="N8" s="14" t="inlineStr">
+        <is>
+          <t>-8%</t>
+        </is>
+      </c>
+      <c r="O8" s="29" t="inlineStr">
+        <is>
+          <t>+47%</t>
+        </is>
+      </c>
+      <c r="P8" s="30" t="inlineStr">
+        <is>
+          <t>+349bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>8/23/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="n">
-        <v>137507207</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>10643451</v>
-      </c>
-      <c r="D9" s="20" t="n">
-        <v>0.07740285932794781</v>
-      </c>
-      <c r="E9" s="18" t="n">
-        <v>132060011</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>10710519</v>
-      </c>
-      <c r="G9" s="20" t="n">
-        <v>0.08110342350342527</v>
-      </c>
-      <c r="H9" s="18" t="n">
-        <v>24881322</v>
-      </c>
-      <c r="I9" s="19" t="n">
-        <v>1911178</v>
-      </c>
-      <c r="J9" s="20" t="n">
-        <v>0.07681175461657544</v>
-      </c>
-      <c r="K9" s="18" t="n">
-        <v>47701558</v>
-      </c>
-      <c r="L9" s="19" t="n">
-        <v>3476356</v>
-      </c>
-      <c r="M9" s="20" t="n">
-        <v>0.07287720036314117</v>
-      </c>
-      <c r="N9" s="18" t="n">
-        <v>381646903</v>
-      </c>
-      <c r="O9" s="19" t="n">
-        <v>30506351</v>
-      </c>
-      <c r="P9" s="20" t="n">
-        <v>0.07993344308626553</v>
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>8/30/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>149527600</v>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>12079306</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>0.08078311963811363</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>146777769</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>15874317</v>
+      </c>
+      <c r="G9" s="23" t="n">
+        <v>0.1081520526449751</v>
+      </c>
+      <c r="H9" s="21" t="n">
+        <v>29155390</v>
+      </c>
+      <c r="I9" s="22" t="n">
+        <v>2727869</v>
+      </c>
+      <c r="J9" s="23" t="n">
+        <v>0.09356311131492324</v>
+      </c>
+      <c r="K9" s="21" t="n">
+        <v>52848942</v>
+      </c>
+      <c r="L9" s="22" t="n">
+        <v>5061346</v>
+      </c>
+      <c r="M9" s="23" t="n">
+        <v>0.09577005344780601</v>
+      </c>
+      <c r="N9" s="21" t="n">
+        <v>420285714</v>
+      </c>
+      <c r="O9" s="22" t="n">
+        <v>39300665</v>
+      </c>
+      <c r="P9" s="23" t="n">
+        <v>0.09350940013154956</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="25" t="inlineStr">
-        <is>
-          <t>+4%</t>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>-10%</t>
         </is>
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>-31%</t>
+          <t>-39%</t>
         </is>
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>-395bps</t>
-        </is>
-      </c>
-      <c r="E10" s="25" t="inlineStr">
-        <is>
-          <t>+5%</t>
+          <t>-392bps</t>
+        </is>
+      </c>
+      <c r="E10" s="28" t="inlineStr">
+        <is>
+          <t>-4%</t>
         </is>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>-4%</t>
+          <t>-27%</t>
         </is>
       </c>
       <c r="G10" s="27" t="inlineStr">
         <is>
-          <t>-78bps</t>
-        </is>
-      </c>
-      <c r="H10" s="22" t="inlineStr">
-        <is>
-          <t>-11%</t>
+          <t>-338bps</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="inlineStr">
+        <is>
+          <t>-25%</t>
         </is>
       </c>
       <c r="I10" s="26" t="inlineStr">
         <is>
-          <t>-36%</t>
+          <t>-37%</t>
         </is>
       </c>
       <c r="J10" s="27" t="inlineStr">
         <is>
-          <t>-301bps</t>
-        </is>
-      </c>
-      <c r="K10" s="22" t="inlineStr">
-        <is>
-          <t>-78%</t>
-        </is>
-      </c>
-      <c r="L10" s="23" t="inlineStr">
-        <is>
-          <t>+688%</t>
-        </is>
-      </c>
-      <c r="M10" s="24" t="inlineStr">
-        <is>
-          <t>+708bps</t>
-        </is>
-      </c>
-      <c r="N10" s="22" t="inlineStr">
-        <is>
-          <t>-30%</t>
+          <t>-186bps</t>
+        </is>
+      </c>
+      <c r="K10" s="28" t="inlineStr">
+        <is>
+          <t>-64%</t>
+        </is>
+      </c>
+      <c r="L10" s="26" t="inlineStr">
+        <is>
+          <t>-66%</t>
+        </is>
+      </c>
+      <c r="M10" s="27" t="inlineStr">
+        <is>
+          <t>-57bps</t>
+        </is>
+      </c>
+      <c r="N10" s="28" t="inlineStr">
+        <is>
+          <t>-25%</t>
         </is>
       </c>
       <c r="O10" s="26" t="inlineStr">
         <is>
-          <t>-11%</t>
-        </is>
-      </c>
-      <c r="P10" s="24" t="inlineStr">
-        <is>
-          <t>+170bps</t>
+          <t>-41%</t>
+        </is>
+      </c>
+      <c r="P10" s="27" t="inlineStr">
+        <is>
+          <t>-259bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>8/16/2026</t>
+          <t>8/23/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>139804782</v>
+        <v>137507207</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>14936414</v>
+        <v>10643451</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>0.1068376473703167</v>
+        <v>0.07740285932794781</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>128334482</v>
+        <v>132060011</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>16567440</v>
+        <v>10710519</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.1290957795738794</v>
+        <v>0.08110342350342527</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>26211607</v>
+        <v>24881322</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>3989974</v>
+        <v>1911178</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.1522216474556482</v>
+        <v>0.07681175461657544</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>43618315</v>
+        <v>47701558</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>4332991</v>
+        <v>3476356</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>0.09933879839237256</v>
+        <v>0.07287720036314117</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>380789208</v>
+        <v>381646903</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>44525193</v>
+        <v>30506351</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>0.1169287155848177</v>
+        <v>0.07993344308626553</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>+14%</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>+38%</t>
-        </is>
-      </c>
-      <c r="D12" s="31" t="inlineStr">
-        <is>
-          <t>+182bps</t>
-        </is>
-      </c>
-      <c r="E12" s="29" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="F12" s="30" t="inlineStr">
-        <is>
-          <t>+17%</t>
-        </is>
-      </c>
-      <c r="G12" s="31" t="inlineStr">
-        <is>
-          <t>+80bps</t>
-        </is>
-      </c>
-      <c r="H12" s="32" t="inlineStr">
-        <is>
-          <t>-1%</t>
-        </is>
-      </c>
-      <c r="I12" s="30" t="inlineStr">
-        <is>
-          <t>+61%</t>
-        </is>
-      </c>
-      <c r="J12" s="31" t="inlineStr">
-        <is>
-          <t>+590bps</t>
-        </is>
-      </c>
-      <c r="K12" s="32" t="inlineStr">
-        <is>
-          <t>-70%</t>
-        </is>
-      </c>
-      <c r="L12" s="30" t="inlineStr">
-        <is>
-          <t>+61%</t>
-        </is>
-      </c>
-      <c r="M12" s="31" t="inlineStr">
-        <is>
-          <t>+811bps</t>
-        </is>
-      </c>
-      <c r="N12" s="32" t="inlineStr">
-        <is>
-          <t>-17%</t>
-        </is>
-      </c>
-      <c r="O12" s="30" t="inlineStr">
-        <is>
-          <t>+34%</t>
-        </is>
-      </c>
-      <c r="P12" s="31" t="inlineStr">
-        <is>
-          <t>+441bps</t>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>+4%</t>
+        </is>
+      </c>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>-31%</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>-395bps</t>
+        </is>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>-4%</t>
+        </is>
+      </c>
+      <c r="G12" s="35" t="inlineStr">
+        <is>
+          <t>-78bps</t>
+        </is>
+      </c>
+      <c r="H12" s="36" t="inlineStr">
+        <is>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="I12" s="34" t="inlineStr">
+        <is>
+          <t>-36%</t>
+        </is>
+      </c>
+      <c r="J12" s="35" t="inlineStr">
+        <is>
+          <t>-301bps</t>
+        </is>
+      </c>
+      <c r="K12" s="36" t="inlineStr">
+        <is>
+          <t>-78%</t>
+        </is>
+      </c>
+      <c r="L12" s="37" t="inlineStr">
+        <is>
+          <t>+688%</t>
+        </is>
+      </c>
+      <c r="M12" s="38" t="inlineStr">
+        <is>
+          <t>+708bps</t>
+        </is>
+      </c>
+      <c r="N12" s="36" t="inlineStr">
+        <is>
+          <t>-30%</t>
+        </is>
+      </c>
+      <c r="O12" s="34" t="inlineStr">
+        <is>
+          <t>-11%</t>
+        </is>
+      </c>
+      <c r="P12" s="38" t="inlineStr">
+        <is>
+          <t>+170bps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NY gaming data - Thu Oct  1 18:00:46 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -817,10 +817,10 @@
         <v>573350554</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>48587565</v>
+        <v>48587566</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.08474320795720379</v>
+        <v>0.08474320930018671</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">

</xml_diff>

<commit_message>
Update NY gaming data - Thu Oct  8 04:00:55 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_weekly_exhibit.xlsx
+++ b/ny_gaming_weekly_exhibit.xlsx
@@ -52,12 +52,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -219,55 +219,64 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -774,53 +783,53 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>9/27/2026</t>
+          <t>10/4/2026</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>196194870</v>
+        <v>213980181</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>18137767</v>
+        <v>13756092</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>0.09244771282755762</v>
+        <v>0.06428675747311383</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>221260979</v>
+        <v>228193108</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>20111002</v>
+        <v>23600001</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>0.09089267385009626</v>
+        <v>0.1034211822032767</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>33450400</v>
+        <v>38130090</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>2799815</v>
+        <v>2671551</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>0.08370049386554421</v>
+        <v>0.07006411471884803</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>64794472</v>
+        <v>70025735</v>
       </c>
       <c r="L3" s="10" t="n">
-        <v>4300521</v>
+        <v>4894277</v>
       </c>
       <c r="M3" s="11" t="n">
-        <v>0.06637172689670193</v>
+        <v>0.06989254736133794</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>573350554</v>
+        <v>619392724</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>48587566</v>
+        <v>49154704</v>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0.08474320930018671</v>
+        <v>0.07935951149468136</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
@@ -831,264 +840,264 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>-2%</t>
+          <t>+1%</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>-22%</t>
+          <t>+82%</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>-234bps</t>
-        </is>
-      </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>+8%</t>
-        </is>
-      </c>
-      <c r="F4" s="17" t="inlineStr">
-        <is>
-          <t>+46%</t>
-        </is>
-      </c>
-      <c r="G4" s="18" t="inlineStr">
-        <is>
-          <t>+236bps</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>-8%</t>
+          <t>+286bps</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>+4%</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>+79%</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>+431bps</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>-6%</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>-34%</t>
+          <t>+7%</t>
         </is>
       </c>
       <c r="J4" s="15" t="inlineStr">
         <is>
-          <t>-341bps</t>
-        </is>
-      </c>
-      <c r="K4" s="16" t="inlineStr">
-        <is>
-          <t>+43%</t>
+          <t>+85bps</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>+44%</t>
         </is>
       </c>
       <c r="L4" s="14" t="inlineStr">
         <is>
-          <t>-4%</t>
+          <t>+101%</t>
         </is>
       </c>
       <c r="M4" s="15" t="inlineStr">
         <is>
-          <t>-322bps</t>
-        </is>
-      </c>
-      <c r="N4" s="16" t="inlineStr">
-        <is>
-          <t>+4%</t>
+          <t>+198bps</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>+5%</t>
         </is>
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>-3%</t>
+          <t>+63%</t>
         </is>
       </c>
       <c r="P4" s="15" t="inlineStr">
         <is>
-          <t>-65bps</t>
+          <t>+283bps</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>9/20/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>208382110</v>
-      </c>
-      <c r="C5" s="21" t="n">
-        <v>14221076</v>
-      </c>
-      <c r="D5" s="22" t="n">
-        <v>0.06824518669093042</v>
-      </c>
-      <c r="E5" s="20" t="n">
-        <v>237685605</v>
-      </c>
-      <c r="F5" s="21" t="n">
-        <v>12919114</v>
-      </c>
-      <c r="G5" s="22" t="n">
-        <v>0.05435379227109694</v>
-      </c>
-      <c r="H5" s="20" t="n">
-        <v>35551693</v>
-      </c>
-      <c r="I5" s="21" t="n">
-        <v>2928353</v>
-      </c>
-      <c r="J5" s="22" t="n">
-        <v>0.08236887621638722</v>
-      </c>
-      <c r="K5" s="20" t="n">
-        <v>70379895</v>
-      </c>
-      <c r="L5" s="21" t="n">
-        <v>4708786</v>
-      </c>
-      <c r="M5" s="22" t="n">
-        <v>0.06690527173989105</v>
-      </c>
-      <c r="N5" s="20" t="n">
-        <v>611081802</v>
-      </c>
-      <c r="O5" s="21" t="n">
-        <v>38507313</v>
-      </c>
-      <c r="P5" s="22" t="n">
-        <v>0.06301498894905727</v>
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>9/27/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>196194870</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>18137767</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <v>0.09244771282755762</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>221260979</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>20111002</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>0.09089267385009626</v>
+      </c>
+      <c r="H5" s="18" t="n">
+        <v>33450400</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>2799815</v>
+      </c>
+      <c r="J5" s="20" t="n">
+        <v>0.08370049386554421</v>
+      </c>
+      <c r="K5" s="18" t="n">
+        <v>64794472</v>
+      </c>
+      <c r="L5" s="19" t="n">
+        <v>4300521</v>
+      </c>
+      <c r="M5" s="20" t="n">
+        <v>0.06637172689670193</v>
+      </c>
+      <c r="N5" s="18" t="n">
+        <v>573350554</v>
+      </c>
+      <c r="O5" s="19" t="n">
+        <v>48587566</v>
+      </c>
+      <c r="P5" s="20" t="n">
+        <v>0.08474320930018671</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>-5%</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="inlineStr">
-        <is>
-          <t>-37%</t>
-        </is>
-      </c>
-      <c r="D6" s="26" t="inlineStr">
-        <is>
-          <t>-339bps</t>
-        </is>
-      </c>
-      <c r="E6" s="27" t="inlineStr">
-        <is>
-          <t>+23%</t>
-        </is>
-      </c>
-      <c r="F6" s="25" t="inlineStr">
-        <is>
-          <t>-46%</t>
-        </is>
-      </c>
-      <c r="G6" s="26" t="inlineStr">
-        <is>
-          <t>-696bps</t>
-        </is>
-      </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>-2%</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>-22%</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>-234bps</t>
+        </is>
+      </c>
+      <c r="E6" s="25" t="inlineStr">
+        <is>
+          <t>+8%</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>+46%</t>
+        </is>
+      </c>
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>+236bps</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>-8%</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>-34%</t>
+        </is>
+      </c>
+      <c r="J6" s="24" t="inlineStr">
+        <is>
+          <t>-341bps</t>
+        </is>
+      </c>
+      <c r="K6" s="25" t="inlineStr">
+        <is>
+          <t>+43%</t>
+        </is>
+      </c>
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>-4%</t>
+        </is>
+      </c>
+      <c r="M6" s="24" t="inlineStr">
+        <is>
+          <t>-322bps</t>
+        </is>
+      </c>
+      <c r="N6" s="25" t="inlineStr">
+        <is>
+          <t>+4%</t>
+        </is>
+      </c>
+      <c r="O6" s="23" t="inlineStr">
         <is>
           <t>-3%</t>
         </is>
       </c>
-      <c r="I6" s="28" t="inlineStr">
-        <is>
-          <t>+45%</t>
-        </is>
-      </c>
-      <c r="J6" s="29" t="inlineStr">
-        <is>
-          <t>+274bps</t>
-        </is>
-      </c>
-      <c r="K6" s="27" t="inlineStr">
-        <is>
-          <t>+57%</t>
-        </is>
-      </c>
-      <c r="L6" s="28" t="inlineStr">
-        <is>
-          <t>+10%</t>
-        </is>
-      </c>
-      <c r="M6" s="26" t="inlineStr">
-        <is>
-          <t>-280bps</t>
-        </is>
-      </c>
-      <c r="N6" s="27" t="inlineStr">
-        <is>
-          <t>+10%</t>
-        </is>
-      </c>
-      <c r="O6" s="25" t="inlineStr">
-        <is>
-          <t>-32%</t>
-        </is>
-      </c>
-      <c r="P6" s="26" t="inlineStr">
-        <is>
-          <t>-394bps</t>
+      <c r="P6" s="24" t="inlineStr">
+        <is>
+          <t>-65bps</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>9/13/2026</t>
+          <t>9/20/2026</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>216744126</v>
+        <v>208382110</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>4743263</v>
+        <v>14221076</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0.02188415938893772</v>
+        <v>0.06824518669093042</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>224469248</v>
+        <v>237685605</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>8347277</v>
+        <v>12919114</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>0.03718672858029978</v>
+        <v>0.05435379227109694</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>35436082</v>
+        <v>35551693</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>966974</v>
+        <v>2928353</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.02728783616653782</v>
+        <v>0.08236887621638722</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>60516979</v>
+        <v>70379895</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>642600</v>
+        <v>4708786</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>0.0106185075761961</v>
+        <v>0.06690527173989105</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>594594280</v>
+        <v>611081802</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>16963073</v>
+        <v>38507313</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.02852881968524823</v>
+        <v>0.06301498894905727</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1099,264 +1108,264 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>+7%</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>-76%</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>-777bps</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>+28%</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>-65%</t>
-        </is>
-      </c>
-      <c r="G8" s="15" t="inlineStr">
-        <is>
-          <t>-1005bps</t>
+          <t>-5%</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>-37%</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>-339bps</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>+23%</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>-46%</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>-696bps</t>
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr">
         <is>
-          <t>+11%</t>
+          <t>-3%</t>
         </is>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
-          <t>-61%</t>
+          <t>+45%</t>
         </is>
       </c>
       <c r="J8" s="15" t="inlineStr">
         <is>
-          <t>-508bps</t>
+          <t>+274bps</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>-8%</t>
+          <t>+57%</t>
         </is>
       </c>
       <c r="L8" s="14" t="inlineStr">
         <is>
-          <t>-88%</t>
-        </is>
-      </c>
-      <c r="M8" s="15" t="inlineStr">
-        <is>
-          <t>-732bps</t>
-        </is>
-      </c>
-      <c r="N8" s="16" t="inlineStr">
-        <is>
-          <t>+11%</t>
-        </is>
-      </c>
-      <c r="O8" s="14" t="inlineStr">
-        <is>
-          <t>-70%</t>
-        </is>
-      </c>
-      <c r="P8" s="15" t="inlineStr">
-        <is>
-          <t>-780bps</t>
+          <t>+10%</t>
+        </is>
+      </c>
+      <c r="M8" s="29" t="inlineStr">
+        <is>
+          <t>-280bps</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
+          <t>+10%</t>
+        </is>
+      </c>
+      <c r="O8" s="28" t="inlineStr">
+        <is>
+          <t>-32%</t>
+        </is>
+      </c>
+      <c r="P8" s="29" t="inlineStr">
+        <is>
+          <t>-394bps</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>9/6/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n">
-        <v>171492780</v>
-      </c>
-      <c r="C9" s="21" t="n">
-        <v>16692306</v>
-      </c>
-      <c r="D9" s="22" t="n">
-        <v>0.0973353280528778</v>
-      </c>
-      <c r="E9" s="20" t="n">
-        <v>167953524</v>
-      </c>
-      <c r="F9" s="21" t="n">
-        <v>16892923</v>
-      </c>
-      <c r="G9" s="22" t="n">
-        <v>0.1005809380933263</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <v>34668902</v>
-      </c>
-      <c r="I9" s="21" t="n">
-        <v>3546293</v>
-      </c>
-      <c r="J9" s="22" t="n">
-        <v>0.1022903177031681</v>
-      </c>
-      <c r="K9" s="20" t="n">
-        <v>56782523</v>
-      </c>
-      <c r="L9" s="21" t="n">
-        <v>3258000</v>
-      </c>
-      <c r="M9" s="22" t="n">
-        <v>0.05737680941017714</v>
-      </c>
-      <c r="N9" s="20" t="n">
-        <v>483313174</v>
-      </c>
-      <c r="O9" s="21" t="n">
-        <v>44849147</v>
-      </c>
-      <c r="P9" s="22" t="n">
-        <v>0.09279520901286253</v>
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>9/13/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>216744126</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>4743263</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>0.02188415938893772</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>224469248</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>8347277</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>0.03718672858029978</v>
+      </c>
+      <c r="H9" s="18" t="n">
+        <v>35436082</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>966974</v>
+      </c>
+      <c r="J9" s="20" t="n">
+        <v>0.02728783616653782</v>
+      </c>
+      <c r="K9" s="18" t="n">
+        <v>60516979</v>
+      </c>
+      <c r="L9" s="19" t="n">
+        <v>642600</v>
+      </c>
+      <c r="M9" s="20" t="n">
+        <v>0.0106185075761961</v>
+      </c>
+      <c r="N9" s="18" t="n">
+        <v>594595202</v>
+      </c>
+      <c r="O9" s="19" t="n">
+        <v>16963507</v>
+      </c>
+      <c r="P9" s="20" t="n">
+        <v>0.02852950535581348</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>yy increase</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>-16%</t>
-        </is>
-      </c>
-      <c r="C10" s="28" t="inlineStr">
-        <is>
-          <t>+273%</t>
-        </is>
-      </c>
-      <c r="D10" s="29" t="inlineStr">
-        <is>
-          <t>+756bps</t>
-        </is>
-      </c>
-      <c r="E10" s="24" t="inlineStr">
-        <is>
-          <t>-3%</t>
-        </is>
-      </c>
-      <c r="F10" s="28" t="inlineStr">
-        <is>
-          <t>+16%</t>
-        </is>
-      </c>
-      <c r="G10" s="29" t="inlineStr">
-        <is>
-          <t>+168bps</t>
-        </is>
-      </c>
-      <c r="H10" s="24" t="inlineStr">
-        <is>
-          <t>-6%</t>
-        </is>
-      </c>
-      <c r="I10" s="28" t="inlineStr">
-        <is>
-          <t>+87%</t>
-        </is>
-      </c>
-      <c r="J10" s="29" t="inlineStr">
-        <is>
-          <t>+509bps</t>
-        </is>
-      </c>
-      <c r="K10" s="27" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="L10" s="25" t="inlineStr">
-        <is>
-          <t>-45%</t>
-        </is>
-      </c>
-      <c r="M10" s="26" t="inlineStr">
-        <is>
-          <t>-567bps</t>
-        </is>
-      </c>
-      <c r="N10" s="24" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>+7%</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>-76%</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>-777bps</t>
+        </is>
+      </c>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>+28%</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>-65%</t>
+        </is>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>-1005bps</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="inlineStr">
+        <is>
+          <t>+11%</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>-61%</t>
+        </is>
+      </c>
+      <c r="J10" s="24" t="inlineStr">
+        <is>
+          <t>-508bps</t>
+        </is>
+      </c>
+      <c r="K10" s="22" t="inlineStr">
         <is>
           <t>-8%</t>
         </is>
       </c>
-      <c r="O10" s="28" t="inlineStr">
-        <is>
-          <t>+47%</t>
-        </is>
-      </c>
-      <c r="P10" s="29" t="inlineStr">
-        <is>
-          <t>+349bps</t>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>-88%</t>
+        </is>
+      </c>
+      <c r="M10" s="24" t="inlineStr">
+        <is>
+          <t>-732bps</t>
+        </is>
+      </c>
+      <c r="N10" s="25" t="inlineStr">
+        <is>
+          <t>+11%</t>
+        </is>
+      </c>
+      <c r="O10" s="23" t="inlineStr">
+        <is>
+          <t>-70%</t>
+        </is>
+      </c>
+      <c r="P10" s="24" t="inlineStr">
+        <is>
+          <t>-780bps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>8/30/2026</t>
+          <t>9/6/2026</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>149527600</v>
+        <v>171492780</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>12079306</v>
+        <v>16692306</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>0.08078311963811363</v>
+        <v>0.0973353280528778</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>146777769</v>
+        <v>167953524</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>15874317</v>
+        <v>16892923</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0.1081520526449751</v>
+        <v>0.1005809380933263</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>29155390</v>
+        <v>34668902</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>2727869</v>
+        <v>3546293</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.09356311131492324</v>
+        <v>0.1022903177031681</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>52848942</v>
+        <v>56782523</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>5061346</v>
+        <v>3258000</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>0.09577005344780601</v>
+        <v>0.05737680941017714</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>420285714</v>
+        <v>483313174</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>39300665</v>
+        <v>44849147</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>0.09350940013154956</v>
+        <v>0.09279520901286253</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -1367,77 +1376,77 @@
       </c>
       <c r="B12" s="31" t="inlineStr">
         <is>
-          <t>-10%</t>
+          <t>-16%</t>
         </is>
       </c>
       <c r="C12" s="32" t="inlineStr">
         <is>
-          <t>-39%</t>
+          <t>+273%</t>
         </is>
       </c>
       <c r="D12" s="33" t="inlineStr">
         <is>
-          <t>-392bps</t>
+          <t>+756bps</t>
         </is>
       </c>
       <c r="E12" s="31" t="inlineStr">
         <is>
-          <t>-4%</t>
+          <t>-3%</t>
         </is>
       </c>
       <c r="F12" s="32" t="inlineStr">
         <is>
-          <t>-27%</t>
+          <t>+16%</t>
         </is>
       </c>
       <c r="G12" s="33" t="inlineStr">
         <is>
-          <t>-338bps</t>
+          <t>+168bps</t>
         </is>
       </c>
       <c r="H12" s="31" t="inlineStr">
         <is>
-          <t>-25%</t>
+          <t>-6%</t>
         </is>
       </c>
       <c r="I12" s="32" t="inlineStr">
         <is>
-          <t>-37%</t>
+          <t>+87%</t>
         </is>
       </c>
       <c r="J12" s="33" t="inlineStr">
         <is>
-          <t>-186bps</t>
-        </is>
-      </c>
-      <c r="K12" s="31" t="inlineStr">
-        <is>
-          <t>-64%</t>
-        </is>
-      </c>
-      <c r="L12" s="32" t="inlineStr">
-        <is>
-          <t>-66%</t>
-        </is>
-      </c>
-      <c r="M12" s="33" t="inlineStr">
-        <is>
-          <t>-57bps</t>
+          <t>+509bps</t>
+        </is>
+      </c>
+      <c r="K12" s="34" t="inlineStr">
+        <is>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="L12" s="35" t="inlineStr">
+        <is>
+          <t>-45%</t>
+        </is>
+      </c>
+      <c r="M12" s="36" t="inlineStr">
+        <is>
+          <t>-567bps</t>
         </is>
       </c>
       <c r="N12" s="31" t="inlineStr">
         <is>
-          <t>-25%</t>
+          <t>-8%</t>
         </is>
       </c>
       <c r="O12" s="32" t="inlineStr">
         <is>
-          <t>-41%</t>
+          <t>+47%</t>
         </is>
       </c>
       <c r="P12" s="33" t="inlineStr">
         <is>
-          <t>-259bps</t>
+          <t>+349bps</t>
         </is>
       </c>
     </row>

</xml_diff>